<commit_message>
week 0 and week 1 - project proposal
</commit_message>
<xml_diff>
--- a/meeting_attendance.xlsx
+++ b/meeting_attendance.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
   <si>
     <t>#</t>
   </si>
@@ -34,46 +34,76 @@
     <t>GABBY</t>
   </si>
   <si>
+    <t>progress made</t>
+  </si>
+  <si>
     <t xml:space="preserve">INITIAL </t>
   </si>
   <si>
-    <t xml:space="preserve">Tuesday Nov 14th </t>
-  </si>
-  <si>
-    <t>From 1:30 PM - 3:00 PM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USC first floor </t>
+    <t xml:space="preserve">Wednsday Nov 15th </t>
+  </si>
+  <si>
+    <t>From 8:00 PM - 9:30 PM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEH study room </t>
   </si>
   <si>
     <t xml:space="preserve">FOR </t>
   </si>
   <si>
-    <t>Saturday Nov 18th</t>
-  </si>
-  <si>
-    <t>From 10:00 AM - 12:00 PM</t>
-  </si>
-  <si>
-    <t>SEH study room</t>
+    <t>Sunday Nov 19th</t>
+  </si>
+  <si>
+    <t>From 10:00 AM - 11:30 PM</t>
+  </si>
+  <si>
+    <t>Zoom Meeting</t>
   </si>
   <si>
     <t>MEETING</t>
   </si>
   <si>
-    <t xml:space="preserve">Monday Nov 20th </t>
-  </si>
-  <si>
-    <t>From 4:00 PM - 5:30 PM</t>
+    <t xml:space="preserve">Sunday Nov 26th </t>
+  </si>
+  <si>
+    <t>From 12:00 PM - 1:00 PM</t>
   </si>
   <si>
     <t>ATTENDANCE</t>
   </si>
   <si>
-    <t>TBD</t>
+    <t xml:space="preserve">Tuesday Nov 28th </t>
+  </si>
+  <si>
+    <t>From 6:00 PM -7:30PM</t>
+  </si>
+  <si>
+    <t>USC First Floor</t>
   </si>
   <si>
     <t>&lt;---------</t>
+  </si>
+  <si>
+    <t>Sunday Nov 3rd</t>
+  </si>
+  <si>
+    <t>From 3:00 PM - 4:00 PM</t>
+  </si>
+  <si>
+    <t>Wednesday Nov 6th</t>
+  </si>
+  <si>
+    <t>Thursday Nov 7th</t>
+  </si>
+  <si>
+    <t>From 7:00 PM - 8:00 PM</t>
+  </si>
+  <si>
+    <t>SEH or Zoom Meeting</t>
+  </si>
+  <si>
+    <t>`</t>
   </si>
 </sst>
 </file>
@@ -205,7 +235,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -228,6 +258,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="8" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -245,8 +278,6 @@
     <xf borderId="1" fillId="12" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="1" fillId="13" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="1" fillId="14" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="1" fillId="10" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="11" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="8" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -493,121 +524,145 @@
       <c r="H1" s="8" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="9" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1">
         <v>1.0</v>
       </c>
-      <c r="B2" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="10" t="s">
+      <c r="B2" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="C2" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="12"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="8" t="s">
+      <c r="D2" s="12" t="s">
         <v>11</v>
+      </c>
+      <c r="E2" s="13"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="15"/>
+      <c r="I2" s="9" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1">
         <v>2.0</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="10" t="s">
+      <c r="B3" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="C3" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="12"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="8" t="s">
+      <c r="D3" s="12" t="s">
         <v>15</v>
+      </c>
+      <c r="E3" s="13"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="15"/>
+      <c r="I3" s="9" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1">
         <v>3.0</v>
       </c>
-      <c r="B4" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="10" t="s">
+      <c r="B4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="12"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="8" t="s">
+      <c r="C4" s="11" t="s">
         <v>18</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="13"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="15"/>
+      <c r="I4" s="9" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1">
         <v>4.0</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="17" t="s">
+      <c r="B5" s="10" t="s">
         <v>20</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="13"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="15"/>
+      <c r="I5" s="16" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1">
         <v>5.0</v>
       </c>
-      <c r="B6" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="14"/>
+      <c r="B6" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="13"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="15"/>
     </row>
     <row r="7">
       <c r="A7" s="1">
         <v>6.0</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="14"/>
+      <c r="B7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="13"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="15"/>
     </row>
     <row r="8">
       <c r="A8" s="1">
         <v>7.0</v>
       </c>
-      <c r="B8" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="14"/>
+      <c r="B8" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="13"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="15"/>
+    </row>
+    <row r="9">
+      <c r="F9" s="8" t="s">
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>